<commit_message>
fix dropdown EditWIF & ChangeExcelForm
</commit_message>
<xml_diff>
--- a/src/Datiss.Budget.Web/wwwroot/excel/WaterInstallFeeImport.xlsx
+++ b/src/Datiss.Budget.Web/wwwroot/excel/WaterInstallFeeImport.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iman\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Budget.Datiss\datiss.budget\src\Datiss.Budget.Web\wwwroot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CE436C-FBDB-459A-AEFE-96860A5A850A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2400" windowWidth="12495" windowHeight="2340"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,22 +27,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>Column1</t>
+    <t>سال</t>
   </si>
   <si>
-    <t>Column2</t>
+    <t>سازمان</t>
   </si>
   <si>
-    <t>Column3</t>
+    <t>کاربری</t>
   </si>
   <si>
-    <t>Column4</t>
+    <t>قیمت</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -92,13 +93,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:D2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="سال"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="سازمان"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="کاربری"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="قیمت"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -366,14 +367,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -387,34 +388,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>890000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>90000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>